<commit_message>
Update Net Profit sensitivity analysis, interactive sliders, and real-time impact indicators
</commit_message>
<xml_diff>
--- a/data/hvn.xlsx
+++ b/data/hvn.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29725"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29822"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://hufiedu-my.sharepoint.com/personal/2046230031_hufi_edu_vn/Documents/phân tích tài chính doanh nghiệp/chương_trình_phân_tich/hvn/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\chương_trình_phân_tich\hvn\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="16" documentId="11_F25DC773A252ABDACC10488E691F44645BDE58E4" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{716F2437-775B-4AB2-9D4F-439AF2886D5B}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{85F6E21E-1456-41E7-90C1-5864385B084B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-13068" yWindow="-4848" windowWidth="13176" windowHeight="22536" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="bs" sheetId="1" r:id="rId1"/>
@@ -18,10 +18,19 @@
     <sheet name="is" sheetId="3" r:id="rId3"/>
     <sheet name="fi" sheetId="4" r:id="rId4"/>
   </sheets>
-  <calcPr calcId="162913"/>
+  <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
+    </ext>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+      </xcalcf:calcFeatures>
     </ext>
   </extLst>
 </workbook>
@@ -1108,6 +1117,7 @@
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="40.54296875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="15.6328125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:16" x14ac:dyDescent="0.35">

</xml_diff>